<commit_message>
Added code to get the data using the upstox api
</commit_message>
<xml_diff>
--- a/refactored_NSE_Automate/ST_calls new.xlsx
+++ b/refactored_NSE_Automate/ST_calls new.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="48">
   <si>
     <t>RowNo</t>
   </si>
@@ -155,6 +155,15 @@
   </si>
   <si>
     <t>SBIN</t>
+  </si>
+  <si>
+    <t>SBIN 920 CE 25 NOV 25</t>
+  </si>
+  <si>
+    <t>instrument_key</t>
+  </si>
+  <si>
+    <t>NSE_FO|117765</t>
   </si>
 </sst>
 </file>
@@ -164,7 +173,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -177,6 +186,14 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -214,7 +231,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -226,6 +243,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -528,16 +546,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T27"/>
+  <dimension ref="A1:U29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="17.77734375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7.88671875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.109375" style="4" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -598,8 +617,11 @@
       <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="U1" s="7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -646,7 +668,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -696,7 +718,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -746,7 +768,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -793,7 +815,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -843,7 +865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -890,7 +912,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -937,7 +959,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -984,7 +1006,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1034,7 +1056,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1081,7 +1103,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1131,7 +1153,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1181,7 +1203,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1228,7 +1250,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1275,7 +1297,7 @@
         <v>91.35</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1322,7 +1344,7 @@
         <v>574.79999999999995</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1372,7 +1394,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1422,7 +1444,7 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1466,7 +1488,7 @@
         <v>758.25</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1516,7 +1538,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1566,7 +1588,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1613,7 +1635,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1660,7 +1682,7 @@
         <v>-8</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1707,7 +1729,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1757,7 +1779,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1807,7 +1829,7 @@
         <v>39.950000000000003</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>25</v>
       </c>
@@ -1857,7 +1879,16 @@
         <v>39.950000000000003</v>
       </c>
     </row>
+    <row r="29" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="G29" t="s">
+        <v>45</v>
+      </c>
+      <c r="U29" t="s">
+        <v>47</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>